<commit_message>
Revert batch parallelism to main; keep summary generation
</commit_message>
<xml_diff>
--- a/batch/tasks_setting.xlsx
+++ b/batch/tasks_setting.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15760"/>
+    <workbookView windowWidth="15488" windowHeight="9317"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Video File</t>
   </si>
@@ -44,28 +44,13 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Parallel</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=c0m6yaGlZh4</t>
+    <t>https://www.youtube.com/watch?v=U4aFbyzrTdc</t>
   </si>
   <si>
     <t>en</t>
   </si>
   <si>
-    <t>zh_CN</t>
-  </si>
-  <si>
-    <t>Error: retry for dubbing</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=vz0UUVDt2ps</t>
-  </si>
-  <si>
-    <t>zh-CN</t>
-  </si>
-  <si>
-    <t>Done</t>
+    <t>French</t>
   </si>
 </sst>
 </file>
@@ -73,10 +58,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -563,7 +548,7 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -572,7 +557,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1059,14 +1044,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="2" outlineLevelCol="5"/>
-  <cols>
-    <col min="1" max="1" width="59.9326923076923" customWidth="1"/>
-    <col min="5" max="5" width="33.9711538461538" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1082,47 +1063,18 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
       <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch: merge per-video summaries; fix align parts mismatch
</commit_message>
<xml_diff>
--- a/batch/tasks_setting.xlsx
+++ b/batch/tasks_setting.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="15488" windowHeight="9317"/>
+    <workbookView windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>Video File</t>
   </si>
@@ -44,13 +44,16 @@
     <t>Status</t>
   </si>
   <si>
-    <t>https://www.youtube.com/watch?v=U4aFbyzrTdc</t>
+    <t>https://www.youtube.com/watch?v=vz0UUVDt2ps</t>
   </si>
   <si>
     <t>en</t>
   </si>
   <si>
-    <t>French</t>
+    <t>简体中文</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=c0m6yaGlZh4</t>
   </si>
 </sst>
 </file>
@@ -58,10 +61,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -548,7 +551,7 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -557,7 +560,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1044,8 +1047,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1" outlineLevelRow="1" outlineLevelCol="4"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="2" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="51.1153846153846" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
@@ -1064,7 +1070,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1075,6 +1081,20 @@
         <v>7</v>
       </c>
       <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3">
         <v>1</v>
       </c>
     </row>

</xml_diff>